<commit_message>
Mejorar identificación de contratistas: columna dedicada en tabla de contratos
Cambios:
- Agregar columna "Contratista" entre "Contrato" y "Subsecretaría" en la pestaña de Contratos
- Mostrar nombre del contratista en negrita con objeto debajo para lectura más rápida
- Ajustar colspan de filas de detalle para mantener alineación
- Regenerar archivos públicos con la nueva estructura de tabla

Resultado: Contratistas ahora son más visibles y fáciles de identificar al revisar el dashboard.
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SECRETARIA_EDUCACION/informes/Seguimiento Presupuestal Educacion a 15_09_2026.xlsx
+++ b/SECRETARIA_EDUCACION/informes/Seguimiento Presupuestal Educacion a 15_09_2026.xlsx
@@ -1155,7 +1155,7 @@
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Fuente: Presupuesto de egreso a 15_09_2026.xls   |   Generado: 2026-09-18   |   Rubros: 127</t>
+          <t>Fuente: Presupuesto de egreso a 15_09_2026.xls   |   Generado: 2026-09-21   |   Rubros: 127</t>
         </is>
       </c>
       <c r="D4" s="5" t="n"/>
@@ -23693,7 +23693,7 @@
       </c>
       <c r="B16" s="87" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>

</xml_diff>